<commit_message>
learning curve analysis updated with Llama3.1 70B
</commit_message>
<xml_diff>
--- a/eval/results/evaluation_metrics.xlsx
+++ b/eval/results/evaluation_metrics.xlsx
@@ -520,19 +520,19 @@
         <v>1920</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9208333333333333</v>
+        <v>0.9213541666666667</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9321329639889196</v>
+        <v>0.9322268326417704</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8672680412371134</v>
+        <v>0.8685567010309279</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8985313751668893</v>
+        <v>0.8992661774516344</v>
       </c>
       <c r="F3" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="G3" t="n">
         <v>1095</v>
@@ -541,7 +541,7 @@
         <v>49</v>
       </c>
       <c r="I3" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -588,19 +588,19 @@
         <v>1920</v>
       </c>
       <c r="B5" t="n">
-        <v>0.79375</v>
+        <v>0.7942708333333334</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7553763440860215</v>
+        <v>0.7557046979865771</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7242268041237113</v>
+        <v>0.7255154639175257</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7394736842105263</v>
+        <v>0.7403024326101247</v>
       </c>
       <c r="F5" t="n">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G5" t="n">
         <v>962</v>
@@ -609,7 +609,7 @@
         <v>182</v>
       </c>
       <c r="I5" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -656,19 +656,19 @@
         <v>1920</v>
       </c>
       <c r="B7" t="n">
-        <v>0.8802083333333334</v>
+        <v>0.8807291666666667</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8719346049046321</v>
+        <v>0.8721088435374149</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8247422680412371</v>
+        <v>0.8260309278350515</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8476821192052979</v>
+        <v>0.8484447385837194</v>
       </c>
       <c r="F7" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="G7" t="n">
         <v>1050</v>
@@ -677,7 +677,7 @@
         <v>94</v>
       </c>
       <c r="I7" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -690,19 +690,19 @@
         <v>1920</v>
       </c>
       <c r="B8" t="n">
-        <v>0.7979166666666667</v>
+        <v>0.7984375</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7957317073170732</v>
+        <v>0.7960426179604262</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6726804123711341</v>
+        <v>0.6739690721649485</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7290502793296091</v>
+        <v>0.7299371946964411</v>
       </c>
       <c r="F8" t="n">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G8" t="n">
         <v>1010</v>
@@ -711,7 +711,7 @@
         <v>134</v>
       </c>
       <c r="I8" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -892,19 +892,19 @@
         <v>1920</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9208333333333333</v>
+        <v>0.9213541666666667</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9321329639889196</v>
+        <v>0.9322268326417704</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8672680412371134</v>
+        <v>0.8685567010309279</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8985313751668893</v>
+        <v>0.8992661774516344</v>
       </c>
       <c r="F3" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="G3" t="n">
         <v>1095</v>
@@ -913,7 +913,7 @@
         <v>49</v>
       </c>
       <c r="I3" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -960,19 +960,19 @@
         <v>1920</v>
       </c>
       <c r="B5" t="n">
-        <v>0.79375</v>
+        <v>0.7942708333333334</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7553763440860215</v>
+        <v>0.7557046979865771</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7242268041237113</v>
+        <v>0.7255154639175257</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7394736842105263</v>
+        <v>0.7403024326101247</v>
       </c>
       <c r="F5" t="n">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G5" t="n">
         <v>962</v>
@@ -981,7 +981,7 @@
         <v>182</v>
       </c>
       <c r="I5" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1028,19 +1028,19 @@
         <v>1920</v>
       </c>
       <c r="B7" t="n">
-        <v>0.8802083333333334</v>
+        <v>0.8807291666666667</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8719346049046321</v>
+        <v>0.8721088435374149</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8247422680412371</v>
+        <v>0.8260309278350515</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8476821192052979</v>
+        <v>0.8484447385837194</v>
       </c>
       <c r="F7" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="G7" t="n">
         <v>1050</v>
@@ -1049,7 +1049,7 @@
         <v>94</v>
       </c>
       <c r="I7" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1062,19 +1062,19 @@
         <v>1920</v>
       </c>
       <c r="B8" t="n">
-        <v>0.7979166666666667</v>
+        <v>0.7984375</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7957317073170732</v>
+        <v>0.7960426179604262</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6726804123711341</v>
+        <v>0.6739690721649485</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7290502793296091</v>
+        <v>0.7299371946964411</v>
       </c>
       <c r="F8" t="n">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G8" t="n">
         <v>1010</v>
@@ -1083,7 +1083,7 @@
         <v>134</v>
       </c>
       <c r="I8" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>

</xml_diff>